<commit_message>
1. Update 5min report template
</commit_message>
<xml_diff>
--- a/report_template/daily5minReport.xlsx
+++ b/report_template/daily5minReport.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repo\Datalogger2\report_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16D7AEB9-BC82-486F-A079-B36F392566CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB92A81D-A41E-4BF3-B2D6-85FAE58B0A2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,28 +33,28 @@
     <t>Date</t>
   </si>
   <si>
-    <t>COD (mg/l)</t>
+    <t>NOx (mg/Nm3)</t>
   </si>
   <si>
-    <t>PH</t>
+    <t>SO2 (mg/Nm3)</t>
   </si>
   <si>
-    <t>TSS (mg/l)</t>
+    <t>Temp (oC)</t>
   </si>
   <si>
-    <t>TEMP (oC)</t>
+    <t>O2 (%)</t>
   </si>
   <si>
-    <t>FLOWOUT (m3/h)</t>
+    <t>Pressure (kPa)</t>
   </si>
   <si>
-    <t>FLOWIN (m3/h)</t>
+    <t>Dust (mg/Nm3)</t>
   </si>
   <si>
-    <t>COLOR (Pt-co)</t>
+    <t>Flow (m3/h)</t>
   </si>
   <si>
-    <t>AMONI (mg/l)</t>
+    <t>CO (mg/Nm3)</t>
   </si>
 </sst>
 </file>

</xml_diff>